<commit_message>
Add new expense tracking files and update existing records in Gitai application. Introduce JSON files for M1 and M2 expenses, along with new PDF documents and images. Increment data snapshot version in config.js for improved data management. Update Excel workbooks to reflect recent changes and enhance overall functionality.
</commit_message>
<xml_diff>
--- a/Gitai-M2.xlsx
+++ b/Gitai-M2.xlsx
@@ -468,7 +468,7 @@
         <v>Gitai.xlsx</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-07-31T14:05:49.559Z</v>
+        <v>2026-07-31T17:48:11.991Z</v>
       </c>
       <c r="E2">
         <v>928</v>
@@ -30924,7 +30924,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>43</v>
+        <v>98</v>
       </c>
       <c r="B2" t="str">
         <v>2022-03-13</v>
@@ -30947,7 +30947,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>73</v>
+        <v>155</v>
       </c>
       <c r="B3" t="str">
         <v>2022-04-23</v>
@@ -30970,7 +30970,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>74</v>
+        <v>156</v>
       </c>
       <c r="B4" t="str">
         <v>2022-04-23</v>
@@ -30993,7 +30993,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>105</v>
+        <v>214</v>
       </c>
       <c r="B5" t="str">
         <v>2022-05-15</v>
@@ -31016,7 +31016,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>119</v>
+        <v>241</v>
       </c>
       <c r="B6" t="str">
         <v>2022-05-28</v>
@@ -31039,7 +31039,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>135</v>
+        <v>273</v>
       </c>
       <c r="B7" t="str">
         <v>2022-06-18</v>
@@ -31062,7 +31062,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>181</v>
+        <v>373</v>
       </c>
       <c r="B8" t="str">
         <v>2023-02-26</v>
@@ -31085,7 +31085,7 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>195</v>
+        <v>398</v>
       </c>
       <c r="B9" t="str">
         <v>2023-04-12</v>
@@ -31108,7 +31108,7 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>199</v>
+        <v>419</v>
       </c>
       <c r="B10" t="str">
         <v>2023-05-15</v>
@@ -31131,7 +31131,7 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>200</v>
+        <v>420</v>
       </c>
       <c r="B11" t="str">
         <v>2023-05-30</v>
@@ -31154,7 +31154,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>201</v>
+        <v>421</v>
       </c>
       <c r="B12" t="str">
         <v>2023-06-18</v>
@@ -31177,7 +31177,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>202</v>
+        <v>422</v>
       </c>
       <c r="B13" t="str">
         <v>2023-06-21</v>
@@ -31200,7 +31200,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>209</v>
+        <v>429</v>
       </c>
       <c r="B14" t="str">
         <v>2023-10-03</v>
@@ -31223,7 +31223,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>212</v>
+        <v>432</v>
       </c>
       <c r="B15" t="str">
         <v>2023-10-17</v>
@@ -31246,7 +31246,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>213</v>
+        <v>433</v>
       </c>
       <c r="B16" t="str">
         <v>2023-10-25</v>
@@ -31269,7 +31269,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>214</v>
+        <v>434</v>
       </c>
       <c r="B17" t="str">
         <v>2023-10-26</v>
@@ -31292,7 +31292,7 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>215</v>
+        <v>435</v>
       </c>
       <c r="B18" t="str">
         <v>2023-10-29</v>
@@ -31315,7 +31315,7 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>216</v>
+        <v>436</v>
       </c>
       <c r="B19" t="str">
         <v>2023-10-30</v>
@@ -31338,7 +31338,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>217</v>
+        <v>438</v>
       </c>
       <c r="B20" t="str">
         <v>2023-11-02</v>
@@ -31361,7 +31361,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>218</v>
+        <v>439</v>
       </c>
       <c r="B21" t="str">
         <v>2023-11-03</v>
@@ -31384,7 +31384,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>219</v>
+        <v>440</v>
       </c>
       <c r="B22" t="str">
         <v>2023-11-11</v>
@@ -31407,7 +31407,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>221</v>
+        <v>442</v>
       </c>
       <c r="B23" t="str">
         <v>2023-11-25</v>
@@ -31430,7 +31430,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>223</v>
+        <v>444</v>
       </c>
       <c r="B24" t="str">
         <v>2023-11-28</v>
@@ -31453,7 +31453,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>233</v>
+        <v>454</v>
       </c>
       <c r="B25" t="str">
         <v>2023-12-10</v>
@@ -31476,7 +31476,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>245</v>
+        <v>466</v>
       </c>
       <c r="B26" t="str">
         <v>2023-12-19</v>
@@ -31499,7 +31499,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>246</v>
+        <v>467</v>
       </c>
       <c r="B27" t="str">
         <v>2023-12-20</v>
@@ -31522,7 +31522,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>247</v>
+        <v>468</v>
       </c>
       <c r="B28" t="str">
         <v>2023-12-21</v>
@@ -31545,7 +31545,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>248</v>
+        <v>469</v>
       </c>
       <c r="B29" t="str">
         <v>2023-12-22</v>
@@ -31568,7 +31568,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>249</v>
+        <v>470</v>
       </c>
       <c r="B30" t="str">
         <v>2023-12-22</v>
@@ -31591,7 +31591,7 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>263</v>
+        <v>484</v>
       </c>
       <c r="B31" t="str">
         <v>2024-01-12</v>
@@ -31614,7 +31614,7 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>264</v>
+        <v>485</v>
       </c>
       <c r="B32" t="str">
         <v>2024-01-15</v>
@@ -31637,7 +31637,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>265</v>
+        <v>486</v>
       </c>
       <c r="B33" t="str">
         <v>2024-01-16</v>
@@ -31660,7 +31660,7 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>293</v>
+        <v>514</v>
       </c>
       <c r="B34" t="str">
         <v>2024-02-12</v>
@@ -31683,7 +31683,7 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>301</v>
+        <v>522</v>
       </c>
       <c r="B35" t="str">
         <v>2024-02-18</v>
@@ -31706,7 +31706,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>303</v>
+        <v>524</v>
       </c>
       <c r="B36" t="str">
         <v>2024-02-24</v>
@@ -31729,7 +31729,7 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>306</v>
+        <v>527</v>
       </c>
       <c r="B37" t="str">
         <v>2024-02-26</v>
@@ -31752,7 +31752,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>307</v>
+        <v>528</v>
       </c>
       <c r="B38" t="str">
         <v>2024-02-27</v>
@@ -31775,7 +31775,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>310</v>
+        <v>531</v>
       </c>
       <c r="B39" t="str">
         <v>2024-02-29</v>
@@ -31798,7 +31798,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>312</v>
+        <v>533</v>
       </c>
       <c r="B40" t="str">
         <v>2024-03-01</v>
@@ -31821,7 +31821,7 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>320</v>
+        <v>541</v>
       </c>
       <c r="B41" t="str">
         <v>2024-03-06</v>
@@ -31844,7 +31844,7 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>322</v>
+        <v>543</v>
       </c>
       <c r="B42" t="str">
         <v>2024-03-12</v>
@@ -31867,7 +31867,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>323</v>
+        <v>544</v>
       </c>
       <c r="B43" t="str">
         <v>2024-03-13</v>
@@ -31890,7 +31890,7 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>324</v>
+        <v>545</v>
       </c>
       <c r="B44" t="str">
         <v>2024-03-13</v>
@@ -31913,7 +31913,7 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>333</v>
+        <v>554</v>
       </c>
       <c r="B45" t="str">
         <v>2024-03-17</v>
@@ -31936,7 +31936,7 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>334</v>
+        <v>555</v>
       </c>
       <c r="B46" t="str">
         <v>2024-03-18</v>
@@ -31959,7 +31959,7 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>335</v>
+        <v>556</v>
       </c>
       <c r="B47" t="str">
         <v>2024-03-23</v>
@@ -31982,7 +31982,7 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>336</v>
+        <v>557</v>
       </c>
       <c r="B48" t="str">
         <v>2024-03-24</v>
@@ -32005,7 +32005,7 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>337</v>
+        <v>558</v>
       </c>
       <c r="B49" t="str">
         <v>2024-03-25</v>
@@ -32028,7 +32028,7 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>338</v>
+        <v>559</v>
       </c>
       <c r="B50" t="str">
         <v>2024-03-28</v>
@@ -32051,7 +32051,7 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>339</v>
+        <v>560</v>
       </c>
       <c r="B51" t="str">
         <v>2024-03-28</v>
@@ -32074,7 +32074,7 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>341</v>
+        <v>562</v>
       </c>
       <c r="B52" t="str">
         <v>2024-04-01</v>
@@ -32097,7 +32097,7 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>345</v>
+        <v>566</v>
       </c>
       <c r="B53" t="str">
         <v>2024-04-02</v>
@@ -32120,7 +32120,7 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>346</v>
+        <v>567</v>
       </c>
       <c r="B54" t="str">
         <v>2024-04-02</v>
@@ -32143,7 +32143,7 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>348</v>
+        <v>569</v>
       </c>
       <c r="B55" t="str">
         <v>2024-04-04</v>
@@ -32166,7 +32166,7 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>352</v>
+        <v>573</v>
       </c>
       <c r="B56" t="str">
         <v>2024-04-06</v>
@@ -32189,7 +32189,7 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>358</v>
+        <v>579</v>
       </c>
       <c r="B57" t="str">
         <v>2024-04-09</v>
@@ -32212,7 +32212,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>361</v>
+        <v>582</v>
       </c>
       <c r="B58" t="str">
         <v>2024-04-10</v>
@@ -32235,7 +32235,7 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>363</v>
+        <v>584</v>
       </c>
       <c r="B59" t="str">
         <v>2024-04-12</v>
@@ -32258,7 +32258,7 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>364</v>
+        <v>585</v>
       </c>
       <c r="B60" t="str">
         <v>2024-04-13</v>
@@ -32281,7 +32281,7 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>366</v>
+        <v>587</v>
       </c>
       <c r="B61" t="str">
         <v>2024-04-17</v>
@@ -32304,7 +32304,7 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>368</v>
+        <v>589</v>
       </c>
       <c r="B62" t="str">
         <v>2024-04-19</v>
@@ -32327,7 +32327,7 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>378</v>
+        <v>599</v>
       </c>
       <c r="B63" t="str">
         <v>2024-04-24</v>
@@ -32350,7 +32350,7 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>392</v>
+        <v>613</v>
       </c>
       <c r="B64" t="str">
         <v>2024-05-04</v>
@@ -32373,7 +32373,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>397</v>
+        <v>618</v>
       </c>
       <c r="B65" t="str">
         <v>2024-05-08</v>
@@ -32396,7 +32396,7 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>411</v>
+        <v>632</v>
       </c>
       <c r="B66" t="str">
         <v>2024-05-14</v>
@@ -32419,7 +32419,7 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>426</v>
+        <v>648</v>
       </c>
       <c r="B67" t="str">
         <v>2024-05-20</v>
@@ -32442,7 +32442,7 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>454</v>
+        <v>676</v>
       </c>
       <c r="B68" t="str">
         <v>2024-05-31</v>
@@ -32465,7 +32465,7 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>465</v>
+        <v>687</v>
       </c>
       <c r="B69" t="str">
         <v>2024-06-02</v>
@@ -32488,7 +32488,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>468</v>
+        <v>690</v>
       </c>
       <c r="B70" t="str">
         <v>2024-06-04</v>
@@ -32511,7 +32511,7 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>492</v>
+        <v>721</v>
       </c>
       <c r="B71" t="str">
         <v>2024-06-24</v>
@@ -32534,7 +32534,7 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>496</v>
+        <v>730</v>
       </c>
       <c r="B72" t="str">
         <v>2024-09-13</v>
@@ -32557,7 +32557,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>504</v>
+        <v>738</v>
       </c>
       <c r="B73" t="str">
         <v>2024-10-08</v>
@@ -32580,7 +32580,7 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>505</v>
+        <v>739</v>
       </c>
       <c r="B74" t="str">
         <v>2024-10-10</v>
@@ -32603,7 +32603,7 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>506</v>
+        <v>740</v>
       </c>
       <c r="B75" t="str">
         <v>2024-10-10</v>
@@ -32626,7 +32626,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>507</v>
+        <v>741</v>
       </c>
       <c r="B76" t="str">
         <v>2024-10-11</v>
@@ -32649,7 +32649,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>508</v>
+        <v>742</v>
       </c>
       <c r="B77" t="str">
         <v>2024-10-23</v>
@@ -32672,7 +32672,7 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>509</v>
+        <v>743</v>
       </c>
       <c r="B78" t="str">
         <v>2024-10-23</v>
@@ -32695,7 +32695,7 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>510</v>
+        <v>744</v>
       </c>
       <c r="B79" t="str">
         <v>2024-11-11</v>
@@ -32718,7 +32718,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>513</v>
+        <v>747</v>
       </c>
       <c r="B80" t="str">
         <v>2024-11-27</v>
@@ -32741,7 +32741,7 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>514</v>
+        <v>748</v>
       </c>
       <c r="B81" t="str">
         <v>2024-11-30</v>
@@ -32764,7 +32764,7 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>515</v>
+        <v>749</v>
       </c>
       <c r="B82" t="str">
         <v>2024-12-01</v>
@@ -32787,7 +32787,7 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>527</v>
+        <v>761</v>
       </c>
       <c r="B83" t="str">
         <v>2024-12-29</v>
@@ -32810,7 +32810,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>538</v>
+        <v>772</v>
       </c>
       <c r="B84" t="str">
         <v>2025-02-21</v>
@@ -32833,7 +32833,7 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>539</v>
+        <v>773</v>
       </c>
       <c r="B85" t="str">
         <v>2025-02-22</v>
@@ -32856,7 +32856,7 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>540</v>
+        <v>774</v>
       </c>
       <c r="B86" t="str">
         <v>2025-03-01</v>
@@ -32879,7 +32879,7 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>546</v>
+        <v>780</v>
       </c>
       <c r="B87" t="str">
         <v>2025-03-10</v>
@@ -32902,7 +32902,7 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>580</v>
+        <v>814</v>
       </c>
       <c r="B88" t="str">
         <v>2025-04-01</v>
@@ -32925,7 +32925,7 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>602</v>
+        <v>836</v>
       </c>
       <c r="B89" t="str">
         <v>2025-04-24</v>
@@ -32948,7 +32948,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>603</v>
+        <v>837</v>
       </c>
       <c r="B90" t="str">
         <v>2025-04-26</v>
@@ -32971,7 +32971,7 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>607</v>
+        <v>841</v>
       </c>
       <c r="B91" t="str">
         <v>2025-04-29</v>
@@ -32994,7 +32994,7 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>612</v>
+        <v>846</v>
       </c>
       <c r="B92" t="str">
         <v>2025-05-01</v>
@@ -33017,7 +33017,7 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>615</v>
+        <v>849</v>
       </c>
       <c r="B93" t="str">
         <v>2025-05-05</v>
@@ -33040,7 +33040,7 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>616</v>
+        <v>850</v>
       </c>
       <c r="B94" t="str">
         <v>2025-05-05</v>
@@ -33063,7 +33063,7 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>617</v>
+        <v>851</v>
       </c>
       <c r="B95" t="str">
         <v>2025-05-05</v>
@@ -33086,7 +33086,7 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>620</v>
+        <v>854</v>
       </c>
       <c r="B96" t="str">
         <v>2025-05-08</v>
@@ -33109,7 +33109,7 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>621</v>
+        <v>855</v>
       </c>
       <c r="B97" t="str">
         <v>2025-05-09</v>
@@ -33132,7 +33132,7 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>622</v>
+        <v>856</v>
       </c>
       <c r="B98" t="str">
         <v>2025-05-10</v>
@@ -33155,7 +33155,7 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>625</v>
+        <v>859</v>
       </c>
       <c r="B99" t="str">
         <v>2025-05-13</v>
@@ -33178,7 +33178,7 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>655</v>
+        <v>889</v>
       </c>
       <c r="B100" t="str">
         <v>2025-07-04</v>
@@ -33201,7 +33201,7 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>656</v>
+        <v>890</v>
       </c>
       <c r="B101" t="str">
         <v>2025-09-01</v>
@@ -33224,7 +33224,7 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>657</v>
+        <v>891</v>
       </c>
       <c r="B102" t="str">
         <v>2025-09-28</v>
@@ -33247,7 +33247,7 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>658</v>
+        <v>892</v>
       </c>
       <c r="B103" t="str">
         <v>2025-11-15</v>
@@ -33270,7 +33270,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>659</v>
+        <v>893</v>
       </c>
       <c r="B104" t="str">
         <v>2025-11-17</v>
@@ -33293,7 +33293,7 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>660</v>
+        <v>894</v>
       </c>
       <c r="B105" t="str">
         <v>2026-02-16</v>
@@ -33316,7 +33316,7 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>661</v>
+        <v>895</v>
       </c>
       <c r="B106" t="str">
         <v>2026-02-16</v>
@@ -33339,7 +33339,7 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>662</v>
+        <v>896</v>
       </c>
       <c r="B107" t="str">
         <v>2026-03-25</v>
@@ -33362,7 +33362,7 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>663</v>
+        <v>897</v>
       </c>
       <c r="B108" t="str">
         <v>2026-05-03</v>
@@ -33385,7 +33385,7 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>664</v>
+        <v>898</v>
       </c>
       <c r="B109" t="str">
         <v>2026-05-06</v>
@@ -33408,7 +33408,7 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>665</v>
+        <v>899</v>
       </c>
       <c r="B110" t="str">
         <v>2026-05-06</v>
@@ -33431,7 +33431,7 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>666</v>
+        <v>900</v>
       </c>
       <c r="B111" t="str">
         <v>2026-05-23</v>
@@ -33454,7 +33454,7 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>667</v>
+        <v>901</v>
       </c>
       <c r="B112" t="str">
         <v>2026-06-01</v>
@@ -33477,7 +33477,7 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>668</v>
+        <v>902</v>
       </c>
       <c r="B113" t="str">
         <v>2026-06-06</v>

</xml_diff>

<commit_message>
Add .DS_Store file and remove temporary Excel file (~$Gitai.xlsx). Update existing Excel workbooks (Gitai-M1.xlsx, Gitai-M2.xlsx, Gitai.xlsx) to reflect recent changes and improve data management.
</commit_message>
<xml_diff>
--- a/Gitai-M2.xlsx
+++ b/Gitai-M2.xlsx
@@ -6343,10 +6343,10 @@
         <v>54400</v>
       </c>
       <c r="H170">
-        <v>34500</v>
+        <v>54400</v>
       </c>
       <c r="I170">
-        <v>19900</v>
+        <v>0</v>
       </c>
       <c r="J170" t="str">
         <v>320 पाईप | जमा 34500 बाकी 19900 | भगवान मुकदम | p16 | imported from Newmachine2.pdf</v>
@@ -9543,10 +9543,10 @@
         <v>75000</v>
       </c>
       <c r="H270">
-        <v>65000</v>
+        <v>75000</v>
       </c>
       <c r="I270">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="J270" t="str">
         <v>10000 बाकी | 498 @150 | p8 | imported from Newmachinevook2.pdf</v>
@@ -9607,10 +9607,10 @@
         <v>47700</v>
       </c>
       <c r="H272">
-        <v>23850</v>
+        <v>41700</v>
       </c>
       <c r="I272">
-        <v>23850</v>
+        <v>6000</v>
       </c>
       <c r="J272" t="str">
         <v>23850 बाकी | 298 ट्रीप @160 | p8 | imported from Newmachinevook2.pdf</v>
@@ -9639,10 +9639,10 @@
         <v>34000</v>
       </c>
       <c r="H273">
-        <v>10000</v>
+        <v>34000</v>
       </c>
       <c r="I273">
-        <v>24000</v>
+        <v>0</v>
       </c>
       <c r="J273" t="str">
         <v>24000 बाकी | 200 ट्रीप @170 | p8 | imported from Newmachinevook2.pdf</v>
@@ -9703,10 +9703,10 @@
         <v>49500</v>
       </c>
       <c r="H275">
-        <v>37000</v>
+        <v>49500</v>
       </c>
       <c r="I275">
-        <v>12500</v>
+        <v>0</v>
       </c>
       <c r="J275" t="str">
         <v>12500 बाकी | 330 @150 | p8 | imported from Newmachinevook2.pdf</v>
@@ -9767,10 +9767,10 @@
         <v>42625</v>
       </c>
       <c r="H277">
-        <v>0</v>
+        <v>42625</v>
       </c>
       <c r="I277">
-        <v>42625</v>
+        <v>0</v>
       </c>
       <c r="J277" t="str">
         <v>42625 बाकी - fully pending | 341 @125 | p8 | imported from Newmachinevook2.pdf</v>
@@ -38405,7 +38405,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J38"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -38441,10 +38441,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-07-31T21:15:10.444Z</v>
+        <v>2026-07-31T21:57:46.558Z</v>
       </c>
       <c r="C2" t="str">
         <v>Administrator</v>
@@ -38453,16 +38453,16 @@
         <v>income</v>
       </c>
       <c r="E2" t="str">
-        <v>UPDATE</v>
+        <v>DELETE</v>
       </c>
       <c r="F2">
-        <v>1767</v>
+        <v>1431</v>
       </c>
       <c r="G2" t="str">
-        <v>{"ID":1767,"Date":"2025-03-25","Customer":"सरपंच ढोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":2.3,"BillAmount":3000,"ReceivedAmount":3000,"PendingAmount":0,"Remarks":"-||- | date assumed from spread/neighbor | 2.30 | p2 | imported from M1_book3_2.pdf"}</v>
+        <v>{"ID":1431,"Date":"2024-05-20","Customer":"Nagorao Barve","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":0,"BillAmount":2520,"ReceivedAmount":0,"PendingAmount":2520,"Remarks":"-||- | date assumed from spread/neighbor | 14 पा | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H2" t="str">
-        <v>{"ID":1767,"Date":"2025-03-25","Customer":"Gajanan Nannaji Dhore","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":2.3,"BillAmount":3000,"ReceivedAmount":3000,"PendingAmount":0,"Remarks":"-||- | date assumed from spread/neighbor | 2.30 | p2 | imported from M1_book3_2.pdf"}</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v>client-side</v>
@@ -38473,10 +38473,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-07-31T21:15:00.639Z</v>
+        <v>2026-07-31T21:57:25.955Z</v>
       </c>
       <c r="C3" t="str">
         <v>Administrator</v>
@@ -38485,16 +38485,16 @@
         <v>income</v>
       </c>
       <c r="E3" t="str">
-        <v>UPDATE</v>
+        <v>DELETE</v>
       </c>
       <c r="F3">
-        <v>1766</v>
+        <v>1430</v>
       </c>
       <c r="G3" t="str">
-        <v>{"ID":1766,"Date":"2025-03-25","Customer":"सरपंच ढोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":38.3,"BillAmount":41800,"ReceivedAmount":0,"PendingAmount":41800,"Remarks":"date assumed from spread/neighbor | 38.30 | p2 | imported from M1_book3_2.pdf"}</v>
+        <v>{"ID":1430,"Date":"2024-05-20","Customer":"Nagorao Barve","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":2.5,"BillAmount":3000,"ReceivedAmount":0,"PendingAmount":3000,"Remarks":"date assumed from spread/neighbor | 2.30 मि | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H3" t="str">
-        <v>{"ID":1766,"Date":"2025-03-25","Customer":"Gajanan Nannaji Dhore","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":38.3,"BillAmount":41800,"ReceivedAmount":41800,"PendingAmount":0,"Remarks":"date assumed from spread/neighbor | 38.30 | p2 | imported from M1_book3_2.pdf"}</v>
+        <v/>
       </c>
       <c r="I3" t="str">
         <v>client-side</v>
@@ -38505,10 +38505,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-07-31T21:14:34.743Z</v>
+        <v>2026-07-31T21:56:56.991Z</v>
       </c>
       <c r="C4" t="str">
         <v>Administrator</v>
@@ -38517,16 +38517,16 @@
         <v>income</v>
       </c>
       <c r="E4" t="str">
-        <v>UPDATE</v>
+        <v>DELETE</v>
       </c>
       <c r="F4">
-        <v>1763</v>
+        <v>1429</v>
       </c>
       <c r="G4" t="str">
-        <v>{"ID":1763,"Date":"2025-03-13","Customer":"सरपंच ढोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":34,"BillAmount":37400,"ReceivedAmount":0,"PendingAmount":37400,"Remarks":"date assumed from spread/neighbor | 34 तास | p1 | imported from M1_book3_2.pdf"}</v>
+        <v>{"ID":1429,"Date":"2024-05-20","Customer":"Vitthal Barve","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":0,"BillAmount":2520,"ReceivedAmount":0,"PendingAmount":2520,"Remarks":"-||- | date assumed from spread/neighbor | 14 पा | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H4" t="str">
-        <v>{"ID":1763,"Date":"2025-03-13","Customer":"Gajanan Nannaji Dhore","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":34,"BillAmount":37400,"ReceivedAmount":37400,"PendingAmount":0,"Remarks":"date assumed from spread/neighbor | 34 तास | p1 | imported from M1_book3_2.pdf"}</v>
+        <v/>
       </c>
       <c r="I4" t="str">
         <v>client-side</v>
@@ -38537,10 +38537,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-07-31T21:13:12.244Z</v>
+        <v>2026-07-31T21:56:45.800Z</v>
       </c>
       <c r="C5" t="str">
         <v>Administrator</v>
@@ -38549,16 +38549,16 @@
         <v>income</v>
       </c>
       <c r="E5" t="str">
-        <v>UPDATE</v>
+        <v>DELETE</v>
       </c>
       <c r="F5">
-        <v>1761</v>
+        <v>1428</v>
       </c>
       <c r="G5" t="str">
-        <v>{"ID":1761,"Date":"2025-03-13","Customer":"सरपंच रोडे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":76.12,"BillAmount":85600,"ReceivedAmount":0,"PendingAmount":85600,"Remarks":"date assumed from spread/neighbor | 76.12 | p1 | imported from M1_book3_2.pdf"}</v>
+        <v>{"ID":1428,"Date":"2024-05-20","Customer":"Vitthal Barve","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":1.5,"BillAmount":1800,"ReceivedAmount":0,"PendingAmount":1800,"Remarks":"-||- | date assumed from spread/neighbor | 1.30 | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H5" t="str">
-        <v>{"ID":1761,"Date":"2025-03-13","Customer":"Gajanan Nannaji Dhore","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":76.12,"BillAmount":85600,"ReceivedAmount":85600,"PendingAmount":0,"Remarks":"date assumed from spread/neighbor | 76.12 | p1 | imported from M1_book3_2.pdf"}</v>
+        <v/>
       </c>
       <c r="I5" t="str">
         <v>client-side</v>
@@ -38569,10 +38569,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-07-31T21:11:19.388Z</v>
+        <v>2026-07-31T21:56:38.143Z</v>
       </c>
       <c r="C6" t="str">
         <v>Administrator</v>
@@ -38581,16 +38581,16 @@
         <v>income</v>
       </c>
       <c r="E6" t="str">
-        <v>UPDATE</v>
+        <v>DELETE</v>
       </c>
       <c r="F6">
-        <v>518</v>
+        <v>1427</v>
       </c>
       <c r="G6" t="str">
-        <v>{"ID":518,"Date":"2023-04-26","Customer":"Ramakant Barve","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":30400,"ReceivedAmount":10000,"PendingAmount":20400,"Remarks":"190 पाईप | जमा 10000 बाकी 20400 | p10 | imported from Newmachine2.pdf"}</v>
+        <v>{"ID":1427,"Date":"2024-05-20","Customer":"Vitthal Barve","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":1.5,"BillAmount":1800,"ReceivedAmount":0,"PendingAmount":1800,"Remarks":"date assumed from spread/neighbor | 1.30 | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H6" t="str">
-        <v>{"ID":518,"Date":"2023-04-26","Customer":"Ramakant Barve","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":30400,"ReceivedAmount":30400,"PendingAmount":0,"Remarks":"190 पाईप | जमा 10000 बाकी 20400 | p10 | imported from Newmachine2.pdf"}</v>
+        <v/>
       </c>
       <c r="I6" t="str">
         <v>client-side</v>
@@ -38601,10 +38601,10 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="B7" t="str">
-        <v>2026-07-31T21:08:42.748Z</v>
+        <v>2026-07-31T21:56:23.449Z</v>
       </c>
       <c r="C7" t="str">
         <v>Administrator</v>
@@ -38613,16 +38613,16 @@
         <v>income</v>
       </c>
       <c r="E7" t="str">
-        <v>UPDATE</v>
+        <v>DELETE</v>
       </c>
       <c r="F7">
-        <v>507</v>
+        <v>1426</v>
       </c>
       <c r="G7" t="str">
-        <v>{"ID":507,"Date":"2023-04-22","Customer":"Shahaji Barve","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":2800,"ReceivedAmount":1800,"PendingAmount":1000,"Remarks":"16 पाईप | 1000 बाकी | p10 | imported from Newmachine2.pdf"}</v>
+        <v>{"ID":1426,"Date":"2024-05-20","Customer":"Rukmaji Barve","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":0,"BillAmount":2520,"ReceivedAmount":0,"PendingAmount":2520,"Remarks":"date assumed from spread/neighbor | 14 पा | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H7" t="str">
-        <v>{"ID":507,"Date":"2023-04-22","Customer":"Shahaji Barve","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":2800,"ReceivedAmount":2800,"PendingAmount":0,"Remarks":"16 पाईप | 1000 बाकी | p10 | imported from Newmachine2.pdf"}</v>
+        <v/>
       </c>
       <c r="I7" t="str">
         <v>client-side</v>
@@ -38633,10 +38633,10 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="B8" t="str">
-        <v>2026-07-31T21:07:23.915Z</v>
+        <v>2026-07-31T21:55:48.044Z</v>
       </c>
       <c r="C8" t="str">
         <v>Administrator</v>
@@ -38648,13 +38648,13 @@
         <v>UPDATE</v>
       </c>
       <c r="F8">
-        <v>372</v>
+        <v>1436</v>
       </c>
       <c r="G8" t="str">
-        <v>{"ID":372,"Date":"2023-02-10","Customer":"Jankiram Tole","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":43,"BillAmount":43000,"ReceivedAmount":8000,"PendingAmount":35000,"Remarks":"43 तास | जमा 8000 बाकी | p3 | imported from Newmachine2.pdf"}</v>
+        <v>{"ID":1436,"Date":"2024-05-20","Customer":"Rambhaji + Hivara Nimbani","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":0,"BillAmount":3000,"ReceivedAmount":0,"PendingAmount":3000,"Remarks":"date assumed from spread/neighbor | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H8" t="str">
-        <v>{"ID":372,"Date":"2023-02-10","Customer":"Jankiram Tole","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":43,"BillAmount":43000,"ReceivedAmount":43000,"PendingAmount":0,"Remarks":"43 तास | जमा 8000 बाकी | p3 | imported from Newmachine2.pdf"}</v>
+        <v>{"ID":1436,"Date":"2024-05-20","Customer":"Rukhmaji","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":0,"BillAmount":3000,"ReceivedAmount":0,"PendingAmount":3000,"Remarks":"date assumed from spread/neighbor | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="I8" t="str">
         <v>client-side</v>
@@ -38665,10 +38665,10 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-07-31T21:05:59.816Z</v>
+        <v>2026-07-31T21:55:12.757Z</v>
       </c>
       <c r="C9" t="str">
         <v>Administrator</v>
@@ -38677,16 +38677,16 @@
         <v>income</v>
       </c>
       <c r="E9" t="str">
-        <v>UPDATE</v>
+        <v>DELETE</v>
       </c>
       <c r="F9">
-        <v>231</v>
+        <v>1425</v>
       </c>
       <c r="G9" t="str">
-        <v>{"ID":231,"Date":"2022-08-17","Customer":"Dhore pralahda &amp; baburao","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"Work hrs","HoursWorked":"","BillAmount":1300,"ReceivedAmount":0,"PendingAmount":1300,"Remarks":"Imported from Gitai_Earthmovers_income-expense-worksheet.xlsx"}</v>
+        <v>{"ID":1425,"Date":"2024-05-20","Customer":"Balubhau Amaik","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":2.5,"BillAmount":3000,"ReceivedAmount":0,"PendingAmount":3000,"Remarks":"-||- | date assumed from spread/neighbor | 2.30 मि | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H9" t="str">
-        <v>{"ID":231,"Date":"2022-08-17","Customer":"Dhore pralahda &amp; baburao","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"Work hrs","HoursWorked":"","BillAmount":2600,"ReceivedAmount":2600,"PendingAmount":0,"Remarks":"Imported from Gitai_Earthmovers_income-expense-worksheet.xlsx"}</v>
+        <v/>
       </c>
       <c r="I9" t="str">
         <v>client-side</v>
@@ -38697,10 +38697,10 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-07-31T21:03:10.905Z</v>
+        <v>2026-07-31T21:54:39.622Z</v>
       </c>
       <c r="C10" t="str">
         <v>Administrator</v>
@@ -38709,16 +38709,16 @@
         <v>income</v>
       </c>
       <c r="E10" t="str">
-        <v>UPDATE</v>
+        <v>DELETE</v>
       </c>
       <c r="F10">
-        <v>66</v>
+        <v>1424</v>
       </c>
       <c r="G10" t="str">
-        <v>{"ID":66,"Date":"2022-03-01","Customer":"baban bepari","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"Trip","HoursWorked":"","BillAmount":4200,"ReceivedAmount":0,"PendingAmount":4200,"Remarks":"Imported from Gitai_Earthmovers_income-expense-worksheet.xlsx"}</v>
+        <v>{"ID":1424,"Date":"2024-05-20","Customer":"Balubhau Amaik","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":1,"BillAmount":1200,"ReceivedAmount":0,"PendingAmount":1200,"Remarks":"-||- | date assumed from spread/neighbor | 1 ता | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H10" t="str">
-        <v>{"ID":66,"Date":"2022-03-01","Customer":"baban bepari","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"Trip","HoursWorked":"","BillAmount":4200,"ReceivedAmount":4200,"PendingAmount":0,"Remarks":"Imported from Gitai_Earthmovers_income-expense-worksheet.xlsx"}</v>
+        <v/>
       </c>
       <c r="I10" t="str">
         <v>client-side</v>
@@ -38729,10 +38729,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-07-31T21:01:59.833Z</v>
+        <v>2026-07-31T21:54:26.958Z</v>
       </c>
       <c r="C11" t="str">
         <v>Administrator</v>
@@ -38741,16 +38741,16 @@
         <v>income</v>
       </c>
       <c r="E11" t="str">
-        <v>UPDATE</v>
+        <v>DELETE</v>
       </c>
       <c r="F11">
-        <v>818</v>
+        <v>1423</v>
       </c>
       <c r="G11" t="str">
-        <v>{"ID":818,"Date":"2023-12-07","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.2,"BillAmount":9900,"ReceivedAmount":0,"PendingAmount":9900,"Remarks":"9 तास 12 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+        <v>{"ID":1423,"Date":"2024-05-20","Customer":"Balubhau Amaik","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":1.5,"BillAmount":1800,"ReceivedAmount":0,"PendingAmount":1800,"Remarks":"-||- | date assumed from spread/neighbor | 1.30 मि | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H11" t="str">
-        <v>{"ID":818,"Date":"2023-12-07","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.2,"BillAmount":9900,"ReceivedAmount":9900,"PendingAmount":0,"Remarks":"9 तास 12 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+        <v/>
       </c>
       <c r="I11" t="str">
         <v>client-side</v>
@@ -38761,10 +38761,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B12" t="str">
-        <v>2026-07-31T21:01:52.442Z</v>
+        <v>2026-07-31T21:54:10.291Z</v>
       </c>
       <c r="C12" t="str">
         <v>Administrator</v>
@@ -38773,16 +38773,16 @@
         <v>income</v>
       </c>
       <c r="E12" t="str">
-        <v>UPDATE</v>
+        <v>DELETE</v>
       </c>
       <c r="F12">
-        <v>821</v>
+        <v>1422</v>
       </c>
       <c r="G12" t="str">
-        <v>{"ID":821,"Date":"2023-12-08","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.3,"BillAmount":10000,"ReceivedAmount":0,"PendingAmount":10000,"Remarks":"9 तास 18 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+        <v>{"ID":1422,"Date":"2024-05-20","Customer":"Balubhau Amaik","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":19,"BillAmount":22800,"ReceivedAmount":0,"PendingAmount":22800,"Remarks":"date assumed from spread/neighbor | 19 तास | p17 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H12" t="str">
-        <v>{"ID":821,"Date":"2023-12-08","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.3,"BillAmount":10000,"ReceivedAmount":10000,"PendingAmount":0,"Remarks":"9 तास 18 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+        <v/>
       </c>
       <c r="I12" t="str">
         <v>client-side</v>
@@ -38793,10 +38793,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="B13" t="str">
-        <v>2026-07-31T21:01:44.216Z</v>
+        <v>2026-07-31T21:46:45.780Z</v>
       </c>
       <c r="C13" t="str">
         <v>Administrator</v>
@@ -38808,13 +38808,13 @@
         <v>UPDATE</v>
       </c>
       <c r="F13">
-        <v>823</v>
+        <v>1014</v>
       </c>
       <c r="G13" t="str">
-        <v>{"ID":823,"Date":"2023-12-09","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":10.5,"BillAmount":11500,"ReceivedAmount":0,"PendingAmount":11500,"Remarks":"10 तास 30 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+        <v>{"ID":1014,"Date":"2024-03-14","Customer":"नान्नाजी ठौरे","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":49500,"ReceivedAmount":37000,"PendingAmount":12500,"Remarks":"12500 बाकी | 330 @150 | p8 | imported from Newmachinevook2.pdf"}</v>
       </c>
       <c r="H13" t="str">
-        <v>{"ID":823,"Date":"2023-12-09","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":10.5,"BillAmount":11500,"ReceivedAmount":11500,"PendingAmount":0,"Remarks":"10 तास 30 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+        <v>{"ID":1014,"Date":"2024-03-14","Customer":"नान्नाजी ठौरे","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":49500,"ReceivedAmount":49500,"PendingAmount":0,"Remarks":"12500 बाकी | 330 @150 | p8 | imported from Newmachinevook2.pdf"}</v>
       </c>
       <c r="I13" t="str">
         <v>client-side</v>
@@ -38825,10 +38825,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="B14" t="str">
-        <v>2026-07-31T21:01:34.108Z</v>
+        <v>2026-07-31T21:46:08.013Z</v>
       </c>
       <c r="C14" t="str">
         <v>Administrator</v>
@@ -38840,13 +38840,13 @@
         <v>UPDATE</v>
       </c>
       <c r="F14">
-        <v>825</v>
+        <v>1009</v>
       </c>
       <c r="G14" t="str">
-        <v>{"ID":825,"Date":"2023-12-10","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.2,"BillAmount":9900,"ReceivedAmount":0,"PendingAmount":9900,"Remarks":"9 तास 12 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+        <v>{"ID":1009,"Date":"2024-03-14","Customer":"वामन ठौरे","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":75000,"ReceivedAmount":65000,"PendingAmount":10000,"Remarks":"10000 बाकी | 498 @150 | p8 | imported from Newmachinevook2.pdf"}</v>
       </c>
       <c r="H14" t="str">
-        <v>{"ID":825,"Date":"2023-12-10","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.2,"BillAmount":9900,"ReceivedAmount":9900,"PendingAmount":0,"Remarks":"9 तास 12 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+        <v>{"ID":1009,"Date":"2024-03-14","Customer":"वामन ठौरे","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":75000,"ReceivedAmount":75000,"PendingAmount":0,"Remarks":"10000 बाकी | 498 @150 | p8 | imported from Newmachinevook2.pdf"}</v>
       </c>
       <c r="I14" t="str">
         <v>client-side</v>
@@ -38857,10 +38857,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="B15" t="str">
-        <v>2026-07-31T21:01:01.499Z</v>
+        <v>2026-07-31T21:45:57.705Z</v>
       </c>
       <c r="C15" t="str">
         <v>Administrator</v>
@@ -38872,13 +38872,13 @@
         <v>UPDATE</v>
       </c>
       <c r="F15">
-        <v>816</v>
+        <v>1011</v>
       </c>
       <c r="G15" t="str">
-        <v>{"ID":816,"Date":"2023-12-06","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":8.3,"BillAmount":9000,"ReceivedAmount":0,"PendingAmount":9000,"Remarks":"8 तास 18 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+        <v>{"ID":1011,"Date":"2024-03-14","Customer":"रंगनाथ अंभोरे","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":47700,"ReceivedAmount":23850,"PendingAmount":23850,"Remarks":"23850 बाकी | 298 ट्रीप @160 | p8 | imported from Newmachinevook2.pdf"}</v>
       </c>
       <c r="H15" t="str">
-        <v>{"ID":816,"Date":"2023-12-06","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":8.3,"BillAmount":9000,"ReceivedAmount":9000,"PendingAmount":0,"Remarks":"8 तास 18 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+        <v>{"ID":1011,"Date":"2024-03-14","Customer":"रंगनाथ अंभोरे","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":47700,"ReceivedAmount":41700,"PendingAmount":6000,"Remarks":"23850 बाकी | 298 ट्रीप @160 | p8 | imported from Newmachinevook2.pdf"}</v>
       </c>
       <c r="I15" t="str">
         <v>client-side</v>
@@ -38889,28 +38889,28 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="B16" t="str">
-        <v>2026-06-13T11:17:08.408Z</v>
+        <v>2026-07-31T21:45:37.855Z</v>
       </c>
       <c r="C16" t="str">
         <v>Administrator</v>
       </c>
       <c r="D16" t="str">
-        <v>partners</v>
+        <v>income</v>
       </c>
       <c r="E16" t="str">
         <v>UPDATE</v>
       </c>
       <c r="F16">
-        <v>3</v>
+        <v>636</v>
       </c>
       <c r="G16" t="str">
-        <v>{"Date":"2023-01-14","PartnerName":"Baliram BArve","TransactionType":"Investment","Amount":100000,"Remarks":"Deposite 2","ID":3}</v>
+        <v>{"ID":636,"Date":"2023-05-23","Customer":"Bhagwan Mukadam","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":54400,"ReceivedAmount":34500,"PendingAmount":19900,"Remarks":"320 पाईप | जमा 34500 बाकी 19900 | भगवान मुकदम | p16 | imported from Newmachine2.pdf"}</v>
       </c>
       <c r="H16" t="str">
-        <v>{"Date":"2023-01-14","PartnerName":"Baliram Barve","TransactionType":"Investment","Amount":100000,"Remarks":"Deposite 2","ID":3}</v>
+        <v>{"ID":636,"Date":"2023-05-23","Customer":"Bhagwan Mukadam","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":54400,"ReceivedAmount":54400,"PendingAmount":0,"Remarks":"320 पाईप | जमा 34500 बाकी 19900 | भगवान मुकदम | p16 | imported from Newmachine2.pdf"}</v>
       </c>
       <c r="I16" t="str">
         <v>client-side</v>
@@ -38921,28 +38921,28 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B17" t="str">
-        <v>2026-06-13T11:17:01.666Z</v>
+        <v>2026-07-31T21:45:22.685Z</v>
       </c>
       <c r="C17" t="str">
         <v>Administrator</v>
       </c>
       <c r="D17" t="str">
-        <v>partners</v>
+        <v>income</v>
       </c>
       <c r="E17" t="str">
         <v>UPDATE</v>
       </c>
       <c r="F17">
-        <v>3</v>
+        <v>1012</v>
       </c>
       <c r="G17" t="str">
-        <v>{"Date":"2023-01-14","PartnerName":"BAliram BArve","TransactionType":"Investment","Amount":100000,"Remarks":"Deposite 2","ID":3}</v>
+        <v>{"ID":1012,"Date":"2024-03-14","Customer":"श्यामा शिंदे","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":34000,"ReceivedAmount":10000,"PendingAmount":24000,"Remarks":"24000 बाकी | 200 ट्रीप @170 | p8 | imported from Newmachinevook2.pdf"}</v>
       </c>
       <c r="H17" t="str">
-        <v>{"Date":"2023-01-14","PartnerName":"Baliram BArve","TransactionType":"Investment","Amount":100000,"Remarks":"Deposite 2","ID":3}</v>
+        <v>{"ID":1012,"Date":"2024-03-14","Customer":"श्यामा शिंदे","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":34000,"ReceivedAmount":34000,"PendingAmount":0,"Remarks":"24000 बाकी | 200 ट्रीप @170 | p8 | imported from Newmachinevook2.pdf"}</v>
       </c>
       <c r="I17" t="str">
         <v>client-side</v>
@@ -38953,28 +38953,28 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-06-13T11:16:38.529Z</v>
+        <v>2026-07-31T21:45:07.647Z</v>
       </c>
       <c r="C18" t="str">
         <v>Administrator</v>
       </c>
       <c r="D18" t="str">
-        <v>partners</v>
+        <v>income</v>
       </c>
       <c r="E18" t="str">
-        <v>CREATE</v>
+        <v>UPDATE</v>
       </c>
       <c r="F18">
-        <v>5</v>
+        <v>1016</v>
       </c>
       <c r="G18" t="str">
-        <v/>
+        <v>{"ID":1016,"Date":"2024-03-14","Customer":"शिवा आबा","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":42625,"ReceivedAmount":0,"PendingAmount":42625,"Remarks":"42625 बाकी - fully pending | 341 @125 | p8 | imported from Newmachinevook2.pdf"}</v>
       </c>
       <c r="H18" t="str">
-        <v>{"Date":"2023-01-14","PartnerName":"Vijay Barve","TransactionType":"Investment","Amount":200000,"Remarks":"Deposite 2","ID":5}</v>
+        <v>{"ID":1016,"Date":"2024-03-14","Customer":"शिवा आबा","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":42625,"ReceivedAmount":42625,"PendingAmount":0,"Remarks":"42625 बाकी - fully pending | 341 @125 | p8 | imported from Newmachinevook2.pdf"}</v>
       </c>
       <c r="I18" t="str">
         <v>client-side</v>
@@ -38985,28 +38985,28 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="B19" t="str">
-        <v>2026-06-13T11:16:14.363Z</v>
+        <v>2026-07-31T21:44:29.263Z</v>
       </c>
       <c r="C19" t="str">
         <v>Administrator</v>
       </c>
       <c r="D19" t="str">
-        <v>partners</v>
+        <v>income</v>
       </c>
       <c r="E19" t="str">
-        <v>CREATE</v>
+        <v>UPDATE</v>
       </c>
       <c r="F19">
-        <v>4</v>
+        <v>1061</v>
       </c>
       <c r="G19" t="str">
-        <v/>
+        <v>{"ID":1061,"Date":"2024-04-01","Customer":"ग्राम पंचायत","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":0,"BillAmount":56000,"ReceivedAmount":25000,"PendingAmount":31000,"Remarks":"जमा 25000 बाकी 31000 | पाईपलाईन 250 B (+ विरार) | p7 | imported from M1_book3_1.pdf"}</v>
       </c>
       <c r="H19" t="str">
-        <v>{"Date":"2022-01-14","PartnerName":"Vijay Barve","TransactionType":"Investment","Amount":250000,"Remarks":"Deposite 1","ID":4}</v>
+        <v>{"ID":1061,"Date":"2024-04-01","Customer":"ग्राम पंचायत","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":0,"BillAmount":56000,"ReceivedAmount":56000,"PendingAmount":0,"Remarks":"जमा 25000 बाकी 31000 | पाईपलाईन 250 B (+ विरार) | p7 | imported from M1_book3_1.pdf"}</v>
       </c>
       <c r="I19" t="str">
         <v>client-side</v>
@@ -39017,28 +39017,28 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>2026-06-13T11:15:30.651Z</v>
+        <v>2026-07-31T21:15:10.444Z</v>
       </c>
       <c r="C20" t="str">
         <v>Administrator</v>
       </c>
       <c r="D20" t="str">
-        <v>partners</v>
+        <v>income</v>
       </c>
       <c r="E20" t="str">
-        <v>CREATE</v>
+        <v>UPDATE</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>1767</v>
       </c>
       <c r="G20" t="str">
-        <v/>
+        <v>{"ID":1767,"Date":"2025-03-25","Customer":"सरपंच ढोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":2.3,"BillAmount":3000,"ReceivedAmount":3000,"PendingAmount":0,"Remarks":"-||- | date assumed from spread/neighbor | 2.30 | p2 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="H20" t="str">
-        <v>{"Date":"2023-01-14","PartnerName":"BAliram BArve","TransactionType":"Investment","Amount":100000,"Remarks":"Deposite 2","ID":3}</v>
+        <v>{"ID":1767,"Date":"2025-03-25","Customer":"Gajanan Nannaji Dhore","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":2.3,"BillAmount":3000,"ReceivedAmount":3000,"PendingAmount":0,"Remarks":"-||- | date assumed from spread/neighbor | 2.30 | p2 | imported from M1_book3_2.pdf"}</v>
       </c>
       <c r="I20" t="str">
         <v>client-side</v>
@@ -39047,9 +39047,585 @@
         <v/>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>18</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-07-31T21:15:00.639Z</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D21" t="str">
+        <v>income</v>
+      </c>
+      <c r="E21" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F21">
+        <v>1766</v>
+      </c>
+      <c r="G21" t="str">
+        <v>{"ID":1766,"Date":"2025-03-25","Customer":"सरपंच ढोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":38.3,"BillAmount":41800,"ReceivedAmount":0,"PendingAmount":41800,"Remarks":"date assumed from spread/neighbor | 38.30 | p2 | imported from M1_book3_2.pdf"}</v>
+      </c>
+      <c r="H21" t="str">
+        <v>{"ID":1766,"Date":"2025-03-25","Customer":"Gajanan Nannaji Dhore","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":38.3,"BillAmount":41800,"ReceivedAmount":41800,"PendingAmount":0,"Remarks":"date assumed from spread/neighbor | 38.30 | p2 | imported from M1_book3_2.pdf"}</v>
+      </c>
+      <c r="I21" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>17</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-07-31T21:14:34.743Z</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D22" t="str">
+        <v>income</v>
+      </c>
+      <c r="E22" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F22">
+        <v>1763</v>
+      </c>
+      <c r="G22" t="str">
+        <v>{"ID":1763,"Date":"2025-03-13","Customer":"सरपंच ढोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":34,"BillAmount":37400,"ReceivedAmount":0,"PendingAmount":37400,"Remarks":"date assumed from spread/neighbor | 34 तास | p1 | imported from M1_book3_2.pdf"}</v>
+      </c>
+      <c r="H22" t="str">
+        <v>{"ID":1763,"Date":"2025-03-13","Customer":"Gajanan Nannaji Dhore","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":34,"BillAmount":37400,"ReceivedAmount":37400,"PendingAmount":0,"Remarks":"date assumed from spread/neighbor | 34 तास | p1 | imported from M1_book3_2.pdf"}</v>
+      </c>
+      <c r="I22" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>16</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-07-31T21:13:12.244Z</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D23" t="str">
+        <v>income</v>
+      </c>
+      <c r="E23" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F23">
+        <v>1761</v>
+      </c>
+      <c r="G23" t="str">
+        <v>{"ID":1761,"Date":"2025-03-13","Customer":"सरपंच रोडे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":76.12,"BillAmount":85600,"ReceivedAmount":0,"PendingAmount":85600,"Remarks":"date assumed from spread/neighbor | 76.12 | p1 | imported from M1_book3_2.pdf"}</v>
+      </c>
+      <c r="H23" t="str">
+        <v>{"ID":1761,"Date":"2025-03-13","Customer":"Gajanan Nannaji Dhore","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":76.12,"BillAmount":85600,"ReceivedAmount":85600,"PendingAmount":0,"Remarks":"date assumed from spread/neighbor | 76.12 | p1 | imported from M1_book3_2.pdf"}</v>
+      </c>
+      <c r="I23" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>15</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-07-31T21:11:19.388Z</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D24" t="str">
+        <v>income</v>
+      </c>
+      <c r="E24" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F24">
+        <v>518</v>
+      </c>
+      <c r="G24" t="str">
+        <v>{"ID":518,"Date":"2023-04-26","Customer":"Ramakant Barve","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":30400,"ReceivedAmount":10000,"PendingAmount":20400,"Remarks":"190 पाईप | जमा 10000 बाकी 20400 | p10 | imported from Newmachine2.pdf"}</v>
+      </c>
+      <c r="H24" t="str">
+        <v>{"ID":518,"Date":"2023-04-26","Customer":"Ramakant Barve","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":30400,"ReceivedAmount":30400,"PendingAmount":0,"Remarks":"190 पाईप | जमा 10000 बाकी 20400 | p10 | imported from Newmachine2.pdf"}</v>
+      </c>
+      <c r="I24" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>14</v>
+      </c>
+      <c r="B25" t="str">
+        <v>2026-07-31T21:08:42.748Z</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D25" t="str">
+        <v>income</v>
+      </c>
+      <c r="E25" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F25">
+        <v>507</v>
+      </c>
+      <c r="G25" t="str">
+        <v>{"ID":507,"Date":"2023-04-22","Customer":"Shahaji Barve","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":2800,"ReceivedAmount":1800,"PendingAmount":1000,"Remarks":"16 पाईप | 1000 बाकी | p10 | imported from Newmachine2.pdf"}</v>
+      </c>
+      <c r="H25" t="str">
+        <v>{"ID":507,"Date":"2023-04-22","Customer":"Shahaji Barve","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":0,"BillAmount":2800,"ReceivedAmount":2800,"PendingAmount":0,"Remarks":"16 पाईप | 1000 बाकी | p10 | imported from Newmachine2.pdf"}</v>
+      </c>
+      <c r="I25" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>13</v>
+      </c>
+      <c r="B26" t="str">
+        <v>2026-07-31T21:07:23.915Z</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D26" t="str">
+        <v>income</v>
+      </c>
+      <c r="E26" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F26">
+        <v>372</v>
+      </c>
+      <c r="G26" t="str">
+        <v>{"ID":372,"Date":"2023-02-10","Customer":"Jankiram Tole","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":43,"BillAmount":43000,"ReceivedAmount":8000,"PendingAmount":35000,"Remarks":"43 तास | जमा 8000 बाकी | p3 | imported from Newmachine2.pdf"}</v>
+      </c>
+      <c r="H26" t="str">
+        <v>{"ID":372,"Date":"2023-02-10","Customer":"Jankiram Tole","Machine":"M2-Mahindra earthmaster sx iv 2023","Site":"","HoursWorked":43,"BillAmount":43000,"ReceivedAmount":43000,"PendingAmount":0,"Remarks":"43 तास | जमा 8000 बाकी | p3 | imported from Newmachine2.pdf"}</v>
+      </c>
+      <c r="I26" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>12</v>
+      </c>
+      <c r="B27" t="str">
+        <v>2026-07-31T21:05:59.816Z</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D27" t="str">
+        <v>income</v>
+      </c>
+      <c r="E27" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F27">
+        <v>231</v>
+      </c>
+      <c r="G27" t="str">
+        <v>{"ID":231,"Date":"2022-08-17","Customer":"Dhore pralahda &amp; baburao","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"Work hrs","HoursWorked":"","BillAmount":1300,"ReceivedAmount":0,"PendingAmount":1300,"Remarks":"Imported from Gitai_Earthmovers_income-expense-worksheet.xlsx"}</v>
+      </c>
+      <c r="H27" t="str">
+        <v>{"ID":231,"Date":"2022-08-17","Customer":"Dhore pralahda &amp; baburao","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"Work hrs","HoursWorked":"","BillAmount":2600,"ReceivedAmount":2600,"PendingAmount":0,"Remarks":"Imported from Gitai_Earthmovers_income-expense-worksheet.xlsx"}</v>
+      </c>
+      <c r="I27" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>11</v>
+      </c>
+      <c r="B28" t="str">
+        <v>2026-07-31T21:03:10.905Z</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D28" t="str">
+        <v>income</v>
+      </c>
+      <c r="E28" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F28">
+        <v>66</v>
+      </c>
+      <c r="G28" t="str">
+        <v>{"ID":66,"Date":"2022-03-01","Customer":"baban bepari","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"Trip","HoursWorked":"","BillAmount":4200,"ReceivedAmount":0,"PendingAmount":4200,"Remarks":"Imported from Gitai_Earthmovers_income-expense-worksheet.xlsx"}</v>
+      </c>
+      <c r="H28" t="str">
+        <v>{"ID":66,"Date":"2022-03-01","Customer":"baban bepari","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"Trip","HoursWorked":"","BillAmount":4200,"ReceivedAmount":4200,"PendingAmount":0,"Remarks":"Imported from Gitai_Earthmovers_income-expense-worksheet.xlsx"}</v>
+      </c>
+      <c r="I28" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>10</v>
+      </c>
+      <c r="B29" t="str">
+        <v>2026-07-31T21:01:59.833Z</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D29" t="str">
+        <v>income</v>
+      </c>
+      <c r="E29" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F29">
+        <v>818</v>
+      </c>
+      <c r="G29" t="str">
+        <v>{"ID":818,"Date":"2023-12-07","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.2,"BillAmount":9900,"ReceivedAmount":0,"PendingAmount":9900,"Remarks":"9 तास 12 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+      </c>
+      <c r="H29" t="str">
+        <v>{"ID":818,"Date":"2023-12-07","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.2,"BillAmount":9900,"ReceivedAmount":9900,"PendingAmount":0,"Remarks":"9 तास 12 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+      </c>
+      <c r="I29" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>9</v>
+      </c>
+      <c r="B30" t="str">
+        <v>2026-07-31T21:01:52.442Z</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D30" t="str">
+        <v>income</v>
+      </c>
+      <c r="E30" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F30">
+        <v>821</v>
+      </c>
+      <c r="G30" t="str">
+        <v>{"ID":821,"Date":"2023-12-08","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.3,"BillAmount":10000,"ReceivedAmount":0,"PendingAmount":10000,"Remarks":"9 तास 18 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+      </c>
+      <c r="H30" t="str">
+        <v>{"ID":821,"Date":"2023-12-08","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.3,"BillAmount":10000,"ReceivedAmount":10000,"PendingAmount":0,"Remarks":"9 तास 18 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+      </c>
+      <c r="I30" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>8</v>
+      </c>
+      <c r="B31" t="str">
+        <v>2026-07-31T21:01:44.216Z</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D31" t="str">
+        <v>income</v>
+      </c>
+      <c r="E31" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F31">
+        <v>823</v>
+      </c>
+      <c r="G31" t="str">
+        <v>{"ID":823,"Date":"2023-12-09","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":10.5,"BillAmount":11500,"ReceivedAmount":0,"PendingAmount":11500,"Remarks":"10 तास 30 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+      </c>
+      <c r="H31" t="str">
+        <v>{"ID":823,"Date":"2023-12-09","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":10.5,"BillAmount":11500,"ReceivedAmount":11500,"PendingAmount":0,"Remarks":"10 तास 30 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+      </c>
+      <c r="I31" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>7</v>
+      </c>
+      <c r="B32" t="str">
+        <v>2026-07-31T21:01:34.108Z</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D32" t="str">
+        <v>income</v>
+      </c>
+      <c r="E32" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F32">
+        <v>825</v>
+      </c>
+      <c r="G32" t="str">
+        <v>{"ID":825,"Date":"2023-12-10","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.2,"BillAmount":9900,"ReceivedAmount":0,"PendingAmount":9900,"Remarks":"9 तास 12 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+      </c>
+      <c r="H32" t="str">
+        <v>{"ID":825,"Date":"2023-12-10","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":9.2,"BillAmount":9900,"ReceivedAmount":9900,"PendingAmount":0,"Remarks":"9 तास 12 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+      </c>
+      <c r="I32" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>6</v>
+      </c>
+      <c r="B33" t="str">
+        <v>2026-07-31T21:01:01.499Z</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D33" t="str">
+        <v>income</v>
+      </c>
+      <c r="E33" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F33">
+        <v>816</v>
+      </c>
+      <c r="G33" t="str">
+        <v>{"ID":816,"Date":"2023-12-06","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":8.3,"BillAmount":9000,"ReceivedAmount":0,"PendingAmount":9000,"Remarks":"8 तास 18 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+      </c>
+      <c r="H33" t="str">
+        <v>{"ID":816,"Date":"2023-12-06","Customer":"आदिनाथ जवन दोरे","Machine":"M1- Mahindra earthmaster sx iv 2022","Site":"","HoursWorked":8.3,"BillAmount":9000,"ReceivedAmount":9000,"PendingAmount":0,"Remarks":"8 तास 18 मि | बाकी | p2 | imported from M1_book3_1.pdf"}</v>
+      </c>
+      <c r="I33" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>5</v>
+      </c>
+      <c r="B34" t="str">
+        <v>2026-06-13T11:17:08.408Z</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D34" t="str">
+        <v>partners</v>
+      </c>
+      <c r="E34" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F34">
+        <v>3</v>
+      </c>
+      <c r="G34" t="str">
+        <v>{"Date":"2023-01-14","PartnerName":"Baliram BArve","TransactionType":"Investment","Amount":100000,"Remarks":"Deposite 2","ID":3}</v>
+      </c>
+      <c r="H34" t="str">
+        <v>{"Date":"2023-01-14","PartnerName":"Baliram Barve","TransactionType":"Investment","Amount":100000,"Remarks":"Deposite 2","ID":3}</v>
+      </c>
+      <c r="I34" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>4</v>
+      </c>
+      <c r="B35" t="str">
+        <v>2026-06-13T11:17:01.666Z</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D35" t="str">
+        <v>partners</v>
+      </c>
+      <c r="E35" t="str">
+        <v>UPDATE</v>
+      </c>
+      <c r="F35">
+        <v>3</v>
+      </c>
+      <c r="G35" t="str">
+        <v>{"Date":"2023-01-14","PartnerName":"BAliram BArve","TransactionType":"Investment","Amount":100000,"Remarks":"Deposite 2","ID":3}</v>
+      </c>
+      <c r="H35" t="str">
+        <v>{"Date":"2023-01-14","PartnerName":"Baliram BArve","TransactionType":"Investment","Amount":100000,"Remarks":"Deposite 2","ID":3}</v>
+      </c>
+      <c r="I35" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>3</v>
+      </c>
+      <c r="B36" t="str">
+        <v>2026-06-13T11:16:38.529Z</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D36" t="str">
+        <v>partners</v>
+      </c>
+      <c r="E36" t="str">
+        <v>CREATE</v>
+      </c>
+      <c r="F36">
+        <v>5</v>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v>{"Date":"2023-01-14","PartnerName":"Vijay Barve","TransactionType":"Investment","Amount":200000,"Remarks":"Deposite 2","ID":5}</v>
+      </c>
+      <c r="I36" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2</v>
+      </c>
+      <c r="B37" t="str">
+        <v>2026-06-13T11:16:14.363Z</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D37" t="str">
+        <v>partners</v>
+      </c>
+      <c r="E37" t="str">
+        <v>CREATE</v>
+      </c>
+      <c r="F37">
+        <v>4</v>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v>{"Date":"2022-01-14","PartnerName":"Vijay Barve","TransactionType":"Investment","Amount":250000,"Remarks":"Deposite 1","ID":4}</v>
+      </c>
+      <c r="I37" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>1</v>
+      </c>
+      <c r="B38" t="str">
+        <v>2026-06-13T11:15:30.651Z</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Administrator</v>
+      </c>
+      <c r="D38" t="str">
+        <v>partners</v>
+      </c>
+      <c r="E38" t="str">
+        <v>CREATE</v>
+      </c>
+      <c r="F38">
+        <v>3</v>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v>{"Date":"2023-01-14","PartnerName":"BAliram BArve","TransactionType":"Investment","Amount":100000,"Remarks":"Deposite 2","ID":3}</v>
+      </c>
+      <c r="I38" t="str">
+        <v>client-side</v>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J38"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>